<commit_message>
Amended the column in the second sheet.
</commit_message>
<xml_diff>
--- a/Dxter_Oring_Analysis_Report.xlsx
+++ b/Dxter_Oring_Analysis_Report.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AmirArshadAbdAziz\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\VSCode\TestDeployment\TestDeployment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3690C890-D7AC-4EED-9387-FA8B1F1B6752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2491C227-1E01-4AA5-BACC-698BE425BD8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="139">
   <si>
     <t>O-RING SPECIFICATION COMPARISON</t>
   </si>
@@ -375,12 +375,6 @@
   </si>
   <si>
     <t>Vendor</t>
-  </si>
-  <si>
-    <t>RFQ Status</t>
-  </si>
-  <si>
-    <t>✔ SEND RFQ</t>
   </si>
   <si>
     <t>Note: Nordvik Sealing AS and TechRubber Europa BV are catalogued as reserve vendors. No RFQ will be issued at this stage due to higher pricing and no existing business relationship.</t>
@@ -465,6 +459,9 @@
   </si>
   <si>
     <t>Email Only</t>
+  </si>
+  <si>
+    <t>Total Weighted Score</t>
   </si>
 </sst>
 </file>
@@ -654,7 +651,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -882,11 +879,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF3A7BD5"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFF0A500"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FFF0A500"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF0A500"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -979,15 +998,6 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1001,6 +1011,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="16" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1016,11 +1032,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1046,10 +1057,25 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1364,41 +1390,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="3" spans="1:8" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
     </row>
     <row r="5" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1454,16 +1480,16 @@
     </row>
     <row r="7" spans="1:8" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="41"/>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="41"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="41"/>
-      <c r="H8" s="41"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1595,58 +1621,58 @@
     </row>
     <row r="14" spans="1:8" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="41"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="41"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="40"/>
+      <c r="E15" s="40"/>
+      <c r="F15" s="40"/>
+      <c r="G15" s="40"/>
+      <c r="H15" s="40"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="51" t="s">
+      <c r="A16" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="52"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="53"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="48"/>
+      <c r="H16" s="49"/>
     </row>
     <row r="17" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="54"/>
-      <c r="B17" s="41"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="41"/>
-      <c r="F17" s="41"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="55"/>
+      <c r="A17" s="50"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="40"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="40"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="51"/>
     </row>
     <row r="18" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="54"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="55"/>
+      <c r="A18" s="50"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="51"/>
     </row>
     <row r="19" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="56"/>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57"/>
-      <c r="D19" s="57"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
-      <c r="H19" s="58"/>
+      <c r="A19" s="52"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="53"/>
+      <c r="D19" s="53"/>
+      <c r="E19" s="53"/>
+      <c r="F19" s="53"/>
+      <c r="G19" s="53"/>
+      <c r="H19" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1674,24 +1700,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="42" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="41" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28"/>
@@ -1700,14 +1726,14 @@
       <c r="D3" s="28"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
     </row>
     <row r="5" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1733,13 +1759,13 @@
       <c r="A6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="61" t="s">
+      <c r="C6" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="61" t="s">
+      <c r="D6" s="37" t="s">
         <v>44</v>
       </c>
       <c r="E6" s="8" t="s">
@@ -1753,13 +1779,13 @@
       <c r="A7" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="61" t="s">
+      <c r="C7" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="61" t="s">
+      <c r="D7" s="37" t="s">
         <v>49</v>
       </c>
       <c r="E7" s="6" t="s">
@@ -1773,13 +1799,13 @@
       <c r="A8" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="61" t="s">
+      <c r="B8" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="C8" s="61" t="s">
+      <c r="C8" s="37" t="s">
         <v>54</v>
       </c>
-      <c r="D8" s="61" t="s">
+      <c r="D8" s="37" t="s">
         <v>55</v>
       </c>
       <c r="E8" s="8" t="s">
@@ -1793,13 +1819,13 @@
       <c r="A9" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="61" t="s">
+      <c r="B9" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="61" t="s">
+      <c r="C9" s="37" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="61" t="s">
+      <c r="D9" s="37" t="s">
         <v>61</v>
       </c>
       <c r="E9" s="6" t="s">
@@ -1813,13 +1839,13 @@
       <c r="A10" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="61" t="s">
+      <c r="C10" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="D10" s="61" t="s">
+      <c r="D10" s="37" t="s">
         <v>65</v>
       </c>
       <c r="E10" s="8" t="s">
@@ -1833,13 +1859,13 @@
       <c r="A11" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="61" t="s">
+      <c r="B11" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="61" t="s">
+      <c r="C11" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="61" t="s">
+      <c r="D11" s="37" t="s">
         <v>70</v>
       </c>
       <c r="E11" s="6" t="s">
@@ -1853,13 +1879,13 @@
       <c r="A12" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="61" t="s">
+      <c r="B12" s="37" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="61" t="s">
+      <c r="C12" s="37" t="s">
         <v>73</v>
       </c>
-      <c r="D12" s="61" t="s">
+      <c r="D12" s="37" t="s">
         <v>72</v>
       </c>
       <c r="E12" s="8" t="s">
@@ -1873,13 +1899,13 @@
       <c r="A13" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B13" s="61" t="s">
+      <c r="B13" s="37" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="61" t="s">
+      <c r="C13" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="D13" s="61" t="s">
+      <c r="D13" s="37" t="s">
         <v>76</v>
       </c>
       <c r="E13" s="6" t="s">
@@ -1893,13 +1919,13 @@
       <c r="A14" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="37" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="61" t="s">
+      <c r="C14" s="37" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="61" t="s">
+      <c r="D14" s="37" t="s">
         <v>82</v>
       </c>
       <c r="E14" s="8" t="s">
@@ -1913,13 +1939,13 @@
       <c r="A15" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="61" t="s">
+      <c r="B15" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="C15" s="61" t="s">
+      <c r="C15" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="D15" s="61" t="s">
+      <c r="D15" s="37" t="s">
         <v>87</v>
       </c>
       <c r="E15" s="6" t="s">
@@ -1933,13 +1959,13 @@
       <c r="A16" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="61" t="s">
+      <c r="B16" s="37" t="s">
         <v>89</v>
       </c>
-      <c r="C16" s="61" t="s">
+      <c r="C16" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="D16" s="61" t="s">
+      <c r="D16" s="37" t="s">
         <v>89</v>
       </c>
       <c r="E16" s="8" t="s">
@@ -1953,33 +1979,33 @@
       <c r="A17" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="61" t="s">
+      <c r="C17" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="D17" s="61" t="s">
+      <c r="D17" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="E17" s="37" t="s">
-        <v>138</v>
-      </c>
-      <c r="F17" s="37" t="s">
-        <v>138</v>
+      <c r="E17" s="34" t="s">
+        <v>136</v>
+      </c>
+      <c r="F17" s="34" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="B18" s="61" t="s">
+      <c r="B18" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="61" t="s">
+      <c r="C18" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="D18" s="61" t="s">
+      <c r="D18" s="37" t="s">
         <v>98</v>
       </c>
       <c r="E18" s="8" t="s">
@@ -1993,13 +2019,13 @@
       <c r="A19" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="D19" s="61" t="s">
+      <c r="D19" s="37" t="s">
         <v>103</v>
       </c>
       <c r="E19" s="6" t="s">
@@ -2013,59 +2039,59 @@
       <c r="A20" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B20" s="61" t="s">
+      <c r="B20" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="C20" s="61" t="s">
+      <c r="C20" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="D20" s="61" t="s">
+      <c r="D20" s="37" t="s">
         <v>106</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="F20" s="38" t="s">
-        <v>139</v>
+      <c r="F20" s="35" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="D21" s="62" t="s">
+      <c r="D21" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="E21" s="37" t="s">
+      <c r="E21" s="34" t="s">
         <v>110</v>
       </c>
-      <c r="F21" s="37" t="s">
+      <c r="F21" s="34" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="B22" s="39">
+        <v>135</v>
+      </c>
+      <c r="B22" s="36">
         <v>4.5</v>
       </c>
-      <c r="C22" s="39">
+      <c r="C22" s="36">
         <v>4</v>
       </c>
-      <c r="D22" s="39">
+      <c r="D22" s="36">
         <v>3.7</v>
       </c>
-      <c r="E22" s="39">
+      <c r="E22" s="36">
         <v>3.3</v>
       </c>
-      <c r="F22" s="39">
+      <c r="F22" s="36">
         <v>3</v>
       </c>
     </row>
@@ -2076,14 +2102,14 @@
       <c r="D23" s="28"/>
     </row>
     <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="40" t="s">
+      <c r="A24" s="60" t="s">
         <v>111</v>
       </c>
-      <c r="B24" s="41"/>
-      <c r="C24" s="41"/>
-      <c r="D24" s="41"/>
-      <c r="E24" s="41"/>
-      <c r="F24" s="41"/>
+      <c r="B24" s="60"/>
+      <c r="C24" s="60"/>
+      <c r="D24" s="60"/>
+      <c r="E24" s="60"/>
+      <c r="F24" s="60"/>
     </row>
     <row r="25" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="29" t="s">
@@ -2102,7 +2128,7 @@
         <v>62</v>
       </c>
       <c r="F25" s="29" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2121,8 +2147,8 @@
       <c r="E26" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="F26" s="32" t="s">
-        <v>114</v>
+      <c r="F26" s="61">
+        <v>4.5</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2141,11 +2167,11 @@
       <c r="E27" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F27" s="33" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F27" s="62">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="12" t="s">
         <v>40</v>
       </c>
@@ -2161,19 +2187,19 @@
       <c r="E28" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F28" s="34" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="45" t="s">
-        <v>115</v>
-      </c>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="47"/>
+      <c r="F28" s="63">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="57" t="s">
+        <v>113</v>
+      </c>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="58"/>
+      <c r="F29" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2204,28 +2230,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
-        <v>116</v>
-      </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
+      <c r="A1" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="42" t="s">
-        <v>117</v>
-      </c>
-      <c r="B2" s="41"/>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="E2" s="41"/>
-      <c r="F2" s="41"/>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
+      <c r="A2" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="3" spans="1:8" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28"/>
@@ -2238,51 +2264,51 @@
       <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
+      <c r="A4" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
     </row>
     <row r="5" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B6" s="15">
         <v>0.2</v>
       </c>
-      <c r="C6" s="35">
+      <c r="C6" s="32">
         <v>4</v>
       </c>
       <c r="D6" s="16">
@@ -2306,12 +2332,12 @@
     </row>
     <row r="7" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B7" s="20">
         <v>0.2</v>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="33">
         <v>5</v>
       </c>
       <c r="D7" s="16">
@@ -2335,12 +2361,12 @@
     </row>
     <row r="8" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B8" s="15">
         <v>0.2</v>
       </c>
-      <c r="C8" s="36">
+      <c r="C8" s="33">
         <v>5</v>
       </c>
       <c r="D8" s="16">
@@ -2369,7 +2395,7 @@
       <c r="B9" s="20">
         <v>0.15</v>
       </c>
-      <c r="C9" s="36">
+      <c r="C9" s="33">
         <v>5</v>
       </c>
       <c r="D9" s="16">
@@ -2393,12 +2419,12 @@
     </row>
     <row r="10" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B10" s="15">
         <v>0.1</v>
       </c>
-      <c r="C10" s="36">
+      <c r="C10" s="33">
         <v>5</v>
       </c>
       <c r="D10" s="16">
@@ -2422,12 +2448,12 @@
     </row>
     <row r="11" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B11" s="20">
         <v>0.05</v>
       </c>
-      <c r="C11" s="36">
+      <c r="C11" s="33">
         <v>5</v>
       </c>
       <c r="D11" s="16">
@@ -2451,12 +2477,12 @@
     </row>
     <row r="12" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B12" s="15">
         <v>0.05</v>
       </c>
-      <c r="C12" s="36">
+      <c r="C12" s="33">
         <v>5</v>
       </c>
       <c r="D12" s="16">
@@ -2480,12 +2506,12 @@
     </row>
     <row r="13" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B13" s="20">
         <v>0.05</v>
       </c>
-      <c r="C13" s="36">
+      <c r="C13" s="33">
         <v>5</v>
       </c>
       <c r="D13" s="16">
@@ -2509,7 +2535,7 @@
     </row>
     <row r="14" spans="1:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="24" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B14" s="25">
         <f t="shared" ref="B14:H14" si="3">SUM(B6:B13)</f>
@@ -2551,68 +2577,68 @@
       <c r="H15" s="28"/>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="40" t="s">
-        <v>135</v>
-      </c>
-      <c r="B16" s="41"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="41"/>
+      <c r="A16" s="39" t="s">
+        <v>133</v>
+      </c>
+      <c r="B16" s="40"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
     </row>
     <row r="17" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="52"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="52"/>
-      <c r="F17" s="52"/>
-      <c r="G17" s="52"/>
-      <c r="H17" s="53"/>
+      <c r="A17" s="56" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" s="48"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
+      <c r="H17" s="49"/>
     </row>
     <row r="18" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="54"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="55"/>
+      <c r="A18" s="50"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="51"/>
     </row>
     <row r="19" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="54"/>
-      <c r="B19" s="41"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="41"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="55"/>
+      <c r="A19" s="50"/>
+      <c r="B19" s="40"/>
+      <c r="C19" s="40"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="40"/>
+      <c r="F19" s="40"/>
+      <c r="G19" s="40"/>
+      <c r="H19" s="51"/>
     </row>
     <row r="20" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="54"/>
-      <c r="B20" s="41"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="41"/>
-      <c r="F20" s="41"/>
-      <c r="G20" s="41"/>
-      <c r="H20" s="55"/>
+      <c r="A20" s="50"/>
+      <c r="B20" s="40"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="40"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="40"/>
+      <c r="H20" s="51"/>
     </row>
     <row r="21" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="56"/>
-      <c r="B21" s="57"/>
-      <c r="C21" s="57"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="57"/>
-      <c r="G21" s="57"/>
-      <c r="H21" s="58"/>
+      <c r="A21" s="52"/>
+      <c r="B21" s="53"/>
+      <c r="C21" s="53"/>
+      <c r="D21" s="53"/>
+      <c r="E21" s="53"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Minor adjustment to the Excel starting page
</commit_message>
<xml_diff>
--- a/Dxter_Oring_Analysis_Report.xlsx
+++ b/Dxter_Oring_Analysis_Report.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2491C227-1E01-4AA5-BACC-698BE425BD8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="O-Ring Comparison" sheetId="1" r:id="rId1"/>
@@ -1019,18 +1019,36 @@
     <xf numFmtId="0" fontId="18" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1054,29 +1072,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1390,41 +1390,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="61" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="44" t="s">
+      <c r="A4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1480,16 +1480,16 @@
     </row>
     <row r="7" spans="1:8" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="44"/>
+      <c r="H8" s="44"/>
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1621,58 +1621,58 @@
     </row>
     <row r="14" spans="1:8" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="45" t="s">
+      <c r="A15" s="51" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="47" t="s">
+      <c r="A16" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="48"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="48"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="48"/>
-      <c r="H16" s="49"/>
+      <c r="B16" s="54"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="54"/>
+      <c r="E16" s="54"/>
+      <c r="F16" s="54"/>
+      <c r="G16" s="54"/>
+      <c r="H16" s="55"/>
     </row>
     <row r="17" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="50"/>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="51"/>
+      <c r="A17" s="56"/>
+      <c r="B17" s="44"/>
+      <c r="C17" s="44"/>
+      <c r="D17" s="44"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="44"/>
+      <c r="H17" s="57"/>
     </row>
     <row r="18" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="50"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="51"/>
+      <c r="A18" s="56"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="57"/>
     </row>
     <row r="19" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="52"/>
-      <c r="B19" s="53"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="54"/>
+      <c r="A19" s="58"/>
+      <c r="B19" s="59"/>
+      <c r="C19" s="59"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="59"/>
+      <c r="F19" s="59"/>
+      <c r="G19" s="59"/>
+      <c r="H19" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1700,24 +1700,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
     </row>
     <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
     </row>
     <row r="3" spans="1:6" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28"/>
@@ -1726,14 +1726,14 @@
       <c r="D3" s="28"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
     </row>
     <row r="5" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -2102,14 +2102,14 @@
       <c r="D23" s="28"/>
     </row>
     <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="60" t="s">
+      <c r="A24" s="42" t="s">
         <v>111</v>
       </c>
-      <c r="B24" s="60"/>
-      <c r="C24" s="60"/>
-      <c r="D24" s="60"/>
-      <c r="E24" s="60"/>
-      <c r="F24" s="60"/>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="42"/>
     </row>
     <row r="25" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="29" t="s">
@@ -2147,7 +2147,7 @@
       <c r="E26" s="31" t="s">
         <v>63</v>
       </c>
-      <c r="F26" s="61">
+      <c r="F26" s="39">
         <v>4.5</v>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       <c r="E27" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F27" s="62">
+      <c r="F27" s="40">
         <v>4</v>
       </c>
     </row>
@@ -2187,19 +2187,19 @@
       <c r="E28" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F28" s="63">
+      <c r="F28" s="41">
         <v>3.7</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="57" t="s">
+      <c r="A29" s="47" t="s">
         <v>113</v>
       </c>
-      <c r="B29" s="58"/>
-      <c r="C29" s="58"/>
-      <c r="D29" s="58"/>
-      <c r="E29" s="58"/>
-      <c r="F29" s="59"/>
+      <c r="B29" s="48"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2230,28 +2230,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="45" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="43" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
     </row>
     <row r="3" spans="1:8" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28"/>
@@ -2264,16 +2264,16 @@
       <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="46" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
+      <c r="H4" s="44"/>
     </row>
     <row r="5" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -2577,68 +2577,68 @@
       <c r="H15" s="28"/>
     </row>
     <row r="16" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="39" t="s">
+      <c r="A16" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="44"/>
+      <c r="H16" s="44"/>
     </row>
     <row r="17" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="56" t="s">
+      <c r="A17" s="63" t="s">
         <v>134</v>
       </c>
-      <c r="B17" s="48"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="48"/>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
-      <c r="G17" s="48"/>
-      <c r="H17" s="49"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="54"/>
+      <c r="H17" s="55"/>
     </row>
     <row r="18" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="50"/>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="51"/>
+      <c r="A18" s="56"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
+      <c r="D18" s="44"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="44"/>
+      <c r="H18" s="57"/>
     </row>
     <row r="19" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="50"/>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="51"/>
+      <c r="A19" s="56"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="44"/>
+      <c r="H19" s="57"/>
     </row>
     <row r="20" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="50"/>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="51"/>
+      <c r="A20" s="56"/>
+      <c r="B20" s="44"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="44"/>
+      <c r="H20" s="57"/>
     </row>
     <row r="21" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="52"/>
-      <c r="B21" s="53"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="53"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="54"/>
+      <c r="A21" s="58"/>
+      <c r="B21" s="59"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
+      <c r="F21" s="59"/>
+      <c r="G21" s="59"/>
+      <c r="H21" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Adjusted where the base selected cell is located
</commit_message>
<xml_diff>
--- a/Dxter_Oring_Analysis_Report.xlsx
+++ b/Dxter_Oring_Analysis_Report.xlsx
@@ -1028,31 +1028,10 @@
     <xf numFmtId="2" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1071,6 +1050,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1390,41 +1390,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:8" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
     </row>
     <row r="5" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -1480,16 +1480,16 @@
     </row>
     <row r="7" spans="1:8" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="44"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="44"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
     </row>
     <row r="9" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
@@ -1621,58 +1621,58 @@
     </row>
     <row r="14" spans="1:8" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="15" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="51" t="s">
+      <c r="A15" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="44"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
-      <c r="H15" s="44"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="43"/>
     </row>
     <row r="16" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="53" t="s">
+      <c r="A16" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="54"/>
-      <c r="C16" s="54"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="54"/>
-      <c r="H16" s="55"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="48"/>
     </row>
     <row r="17" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="56"/>
-      <c r="B17" s="44"/>
-      <c r="C17" s="44"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="57"/>
+      <c r="A17" s="49"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="43"/>
+      <c r="G17" s="43"/>
+      <c r="H17" s="50"/>
     </row>
     <row r="18" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="56"/>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="44"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="57"/>
+      <c r="A18" s="49"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="50"/>
     </row>
     <row r="19" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="58"/>
-      <c r="B19" s="59"/>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="59"/>
-      <c r="F19" s="59"/>
-      <c r="G19" s="59"/>
-      <c r="H19" s="60"/>
+      <c r="A19" s="51"/>
+      <c r="B19" s="52"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1700,24 +1700,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
     </row>
     <row r="2" spans="1:6" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="56" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
     </row>
     <row r="3" spans="1:6" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28"/>
@@ -1726,14 +1726,14 @@
       <c r="D3" s="28"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
     </row>
     <row r="5" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -2102,14 +2102,14 @@
       <c r="D23" s="28"/>
     </row>
     <row r="24" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="42" t="s">
+      <c r="A24" s="55" t="s">
         <v>111</v>
       </c>
-      <c r="B24" s="42"/>
-      <c r="C24" s="42"/>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="42"/>
+      <c r="B24" s="55"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
     </row>
     <row r="25" spans="1:6" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="29" t="s">
@@ -2192,14 +2192,14 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="47" t="s">
+      <c r="A29" s="59" t="s">
         <v>113</v>
       </c>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="49"/>
+      <c r="B29" s="60"/>
+      <c r="C29" s="60"/>
+      <c r="D29" s="60"/>
+      <c r="E29" s="60"/>
+      <c r="F29" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2230,28 +2230,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="57" t="s">
         <v>114</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
     </row>
     <row r="2" spans="1:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="56" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="44"/>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
     </row>
     <row r="3" spans="1:8" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="28"/>
@@ -2264,16 +2264,16 @@
       <c r="H3" s="28"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="58" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="44"/>
-      <c r="F4" s="44"/>
-      <c r="G4" s="44"/>
-      <c r="H4" s="44"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="43"/>
     </row>
     <row r="5" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -2580,65 +2580,65 @@
       <c r="A16" s="62" t="s">
         <v>133</v>
       </c>
-      <c r="B16" s="44"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="44"/>
-      <c r="H16" s="44"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="43"/>
     </row>
     <row r="17" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="63" t="s">
         <v>134</v>
       </c>
-      <c r="B17" s="54"/>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54"/>
-      <c r="G17" s="54"/>
-      <c r="H17" s="55"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="47"/>
+      <c r="G17" s="47"/>
+      <c r="H17" s="48"/>
     </row>
     <row r="18" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="56"/>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="44"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="57"/>
+      <c r="A18" s="49"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="50"/>
     </row>
     <row r="19" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="56"/>
-      <c r="B19" s="44"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="44"/>
-      <c r="G19" s="44"/>
-      <c r="H19" s="57"/>
+      <c r="A19" s="49"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="50"/>
     </row>
     <row r="20" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="56"/>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="44"/>
-      <c r="F20" s="44"/>
-      <c r="G20" s="44"/>
-      <c r="H20" s="57"/>
+      <c r="A20" s="49"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="50"/>
     </row>
     <row r="21" spans="1:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="58"/>
-      <c r="B21" s="59"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="59"/>
-      <c r="E21" s="59"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="59"/>
-      <c r="H21" s="60"/>
+      <c r="A21" s="51"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>